<commit_message>
add NHS hospital cost plan budget figures - £18M total
</commit_message>
<xml_diff>
--- a/cost-plans/NHS-Acute-Hospital-Wing.xlsx
+++ b/cost-plans/NHS-Acute-Hospital-Wing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE73F58D-85B7-4246-85E2-0B1BAAEC13FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5347167-034D-4AD2-8A5B-C306EB7BE88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
@@ -281,7 +281,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -299,6 +299,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E5496"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -313,19 +331,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -336,8 +367,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF1F3864"/>
+      <color rgb="FFD9D9D9"/>
       <color rgb="FF2E5496"/>
-      <color rgb="FF1F3864"/>
     </mruColors>
   </colors>
   <extLst>
@@ -666,12 +698,34 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="613" row="5">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{E3ADDD4B-ED9F-435E-AC38-9852B6340747}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;ce0ff0a3-417f-49c5-a90f-eb41d57900c7&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B8CA9C0-9C58-4F75-869D-8D1A35F325AC}">
   <dimension ref="A1:J27"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.69140625" style="5" customWidth="1"/>
+    <col min="1" max="1" width="12.69140625" style="4" customWidth="1"/>
     <col min="2" max="2" width="35.69140625" customWidth="1"/>
     <col min="3" max="3" width="16.69140625" customWidth="1"/>
     <col min="4" max="4" width="20.69140625" customWidth="1"/>
@@ -682,245 +736,429 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>47</v>
       </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="8" t="s">
         <v>48</v>
       </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="9" t="s">
         <v>49</v>
       </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="6" t="s">
         <v>50</v>
       </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="8" t="s">
         <v>51</v>
       </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="9" t="s">
         <v>52</v>
       </c>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="8" t="s">
         <v>53</v>
       </c>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="8" t="s">
         <v>55</v>
       </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="9" t="s">
         <v>56</v>
       </c>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="6" t="s">
         <v>57</v>
       </c>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="8" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A17" s="5" t="s">
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A17" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A18" s="5" t="s">
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A18" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A19" s="5" t="s">
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A19" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="6" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A20" s="5" t="s">
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A20" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="6" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A21" s="5" t="s">
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A21" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="8" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A22" s="5" t="s">
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A22" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="9" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A23" s="5" t="s">
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A23" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="8" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A24" s="5" t="s">
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A24" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="6" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A25" s="5" t="s">
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="6"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A25" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="6" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A26" s="5" t="s">
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="A26" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="6" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="B27" t="s">
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="B27" s="7" t="s">
         <v>69</v>
       </c>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
add committed, actual, EAC, variance and % complete columns to NHS cost plan
</commit_message>
<xml_diff>
--- a/cost-plans/NHS-Acute-Hospital-Wing.xlsx
+++ b/cost-plans/NHS-Acute-Hospital-Wing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5347167-034D-4AD2-8A5B-C306EB7BE88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3638E78-CF86-4C36-84C9-D74999CBBF7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
@@ -257,7 +257,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -276,6 +276,13 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -327,11 +334,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -358,10 +366,19 @@
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="1" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="2" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -802,14 +819,35 @@
       <c r="B5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
+      <c r="C5" s="6">
+        <f>SUM(C6:C7)</f>
+        <v>800000</v>
+      </c>
+      <c r="D5" s="14"/>
+      <c r="E5" s="6">
+        <f>SUM(C5:D5)</f>
+        <v>800000</v>
+      </c>
+      <c r="F5" s="6">
+        <f>SUM(F6:F7)</f>
+        <v>800000</v>
+      </c>
+      <c r="G5" s="6">
+        <f>SUM(G6:G7)</f>
+        <v>720000</v>
+      </c>
+      <c r="H5" s="6">
+        <f>SUM(H6:H7)</f>
+        <v>805000</v>
+      </c>
+      <c r="I5" s="6">
+        <f>E5-H5</f>
+        <v>-5000</v>
+      </c>
+      <c r="J5" s="18">
+        <f>SUMPRODUCT(E6:E7, J6:J7)/SUM(E6:E7)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A6" s="12" t="s">
@@ -818,14 +856,30 @@
       <c r="B6" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
+      <c r="C6" s="8">
+        <v>540000</v>
+      </c>
+      <c r="D6" s="15"/>
+      <c r="E6" s="8">
+        <f t="shared" ref="E6:F26" si="0">SUM(C6:D6)</f>
+        <v>540000</v>
+      </c>
+      <c r="F6" s="8">
+        <v>540000</v>
+      </c>
+      <c r="G6" s="8">
+        <v>486000</v>
+      </c>
+      <c r="H6" s="8">
+        <v>540000</v>
+      </c>
+      <c r="I6" s="8">
+        <f t="shared" ref="I6:I27" si="1">E6-H6</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A7" s="13" t="s">
@@ -834,14 +888,30 @@
       <c r="B7" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
+      <c r="C7" s="9">
+        <v>260000</v>
+      </c>
+      <c r="D7" s="16"/>
+      <c r="E7" s="9">
+        <f t="shared" si="0"/>
+        <v>260000</v>
+      </c>
+      <c r="F7" s="9">
+        <v>260000</v>
+      </c>
+      <c r="G7" s="9">
+        <v>234000</v>
+      </c>
+      <c r="H7" s="9">
+        <v>265000</v>
+      </c>
+      <c r="I7" s="9">
+        <f t="shared" si="1"/>
+        <v>-5000</v>
+      </c>
+      <c r="J7" s="20">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A8" s="11" t="s">
@@ -850,14 +920,38 @@
       <c r="B8" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
+      <c r="C8" s="6">
+        <f>SUM(C9:C14)</f>
+        <v>4290000</v>
+      </c>
+      <c r="D8" s="14">
+        <f>SUM(D9:D14)</f>
+        <v>45000</v>
+      </c>
+      <c r="E8" s="6">
+        <f t="shared" si="0"/>
+        <v>4335000</v>
+      </c>
+      <c r="F8" s="6">
+        <f>SUM(F9:F14)</f>
+        <v>4121000</v>
+      </c>
+      <c r="G8" s="6">
+        <f>SUM(G9:G14)</f>
+        <v>3708950</v>
+      </c>
+      <c r="H8" s="6">
+        <f>SUM(H9:H14)</f>
+        <v>4315000</v>
+      </c>
+      <c r="I8" s="6">
+        <f t="shared" si="1"/>
+        <v>20000</v>
+      </c>
+      <c r="J8" s="18">
+        <f>SUMPRODUCT(E9:E14,J9:J14)/SUM(E9:E14)</f>
+        <v>0.92612456747404848</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A9" s="12" t="s">
@@ -866,14 +960,30 @@
       <c r="B9" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="C9" s="8">
+        <v>1800000</v>
+      </c>
+      <c r="D9" s="15"/>
+      <c r="E9" s="8">
+        <f t="shared" si="0"/>
+        <v>1800000</v>
+      </c>
+      <c r="F9" s="8">
+        <v>1800000</v>
+      </c>
+      <c r="G9" s="8">
+        <v>1620000</v>
+      </c>
+      <c r="H9" s="8">
+        <v>1800000</v>
+      </c>
+      <c r="I9" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="19">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A10" s="13" t="s">
@@ -882,14 +992,30 @@
       <c r="B10" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
+      <c r="C10" s="9">
+        <v>650000</v>
+      </c>
+      <c r="D10" s="16"/>
+      <c r="E10" s="9">
+        <f t="shared" si="0"/>
+        <v>650000</v>
+      </c>
+      <c r="F10" s="9">
+        <v>650000</v>
+      </c>
+      <c r="G10" s="9">
+        <v>585000</v>
+      </c>
+      <c r="H10" s="9">
+        <v>650000</v>
+      </c>
+      <c r="I10" s="9">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J10" s="20">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A11" s="12" t="s">
@@ -898,14 +1024,30 @@
       <c r="B11" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="C11" s="8">
+        <v>280000</v>
+      </c>
+      <c r="D11" s="15"/>
+      <c r="E11" s="8">
+        <f t="shared" si="0"/>
+        <v>280000</v>
+      </c>
+      <c r="F11" s="8">
+        <v>266000</v>
+      </c>
+      <c r="G11" s="8">
+        <v>239400</v>
+      </c>
+      <c r="H11" s="8">
+        <v>272000</v>
+      </c>
+      <c r="I11" s="8">
+        <f t="shared" si="1"/>
+        <v>8000</v>
+      </c>
+      <c r="J11" s="19">
+        <v>0.95</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A12" s="13" t="s">
@@ -914,14 +1056,32 @@
       <c r="B12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
+      <c r="C12" s="9">
+        <v>950000</v>
+      </c>
+      <c r="D12" s="16">
+        <v>45000</v>
+      </c>
+      <c r="E12" s="9">
+        <f t="shared" si="0"/>
+        <v>995000</v>
+      </c>
+      <c r="F12" s="9">
+        <v>895500</v>
+      </c>
+      <c r="G12" s="9">
+        <v>806000</v>
+      </c>
+      <c r="H12" s="9">
+        <v>1045000</v>
+      </c>
+      <c r="I12" s="9">
+        <f t="shared" si="1"/>
+        <v>-50000</v>
+      </c>
+      <c r="J12" s="20">
+        <v>0.85</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A13" s="12" t="s">
@@ -930,14 +1090,30 @@
       <c r="B13" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
+      <c r="C13" s="8">
+        <v>520000</v>
+      </c>
+      <c r="D13" s="15"/>
+      <c r="E13" s="8">
+        <f t="shared" si="0"/>
+        <v>520000</v>
+      </c>
+      <c r="F13" s="8">
+        <v>442000</v>
+      </c>
+      <c r="G13" s="8">
+        <v>397800</v>
+      </c>
+      <c r="H13" s="8">
+        <v>476000</v>
+      </c>
+      <c r="I13" s="8">
+        <f t="shared" si="1"/>
+        <v>44000</v>
+      </c>
+      <c r="J13" s="19">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A14" s="13" t="s">
@@ -946,14 +1122,30 @@
       <c r="B14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
+      <c r="C14" s="9">
+        <v>90000</v>
+      </c>
+      <c r="D14" s="16"/>
+      <c r="E14" s="9">
+        <f t="shared" si="0"/>
+        <v>90000</v>
+      </c>
+      <c r="F14" s="9">
+        <v>67500</v>
+      </c>
+      <c r="G14" s="9">
+        <v>60750</v>
+      </c>
+      <c r="H14" s="9">
+        <v>72000</v>
+      </c>
+      <c r="I14" s="9">
+        <f t="shared" si="1"/>
+        <v>18000</v>
+      </c>
+      <c r="J14" s="20">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A15" s="11" t="s">
@@ -962,14 +1154,38 @@
       <c r="B15" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
+      <c r="C15" s="6">
+        <f>SUM(C16:C18)</f>
+        <v>790000</v>
+      </c>
+      <c r="D15" s="14">
+        <f>SUM(D16:D18)</f>
+        <v>28000</v>
+      </c>
+      <c r="E15" s="6">
+        <f t="shared" si="0"/>
+        <v>818000</v>
+      </c>
+      <c r="F15" s="6">
+        <f>SUM(F16:F18)</f>
+        <v>626500</v>
+      </c>
+      <c r="G15" s="6">
+        <f>SUM(G16:G18)</f>
+        <v>501200</v>
+      </c>
+      <c r="H15" s="6">
+        <f>SUM(H16:H18)</f>
+        <v>842000</v>
+      </c>
+      <c r="I15" s="6">
+        <f t="shared" si="1"/>
+        <v>-24000</v>
+      </c>
+      <c r="J15" s="18">
+        <f>SUMPRODUCT(E16:E18,J16:J18)/SUM(E16:E18)</f>
+        <v>0.61589242053789728</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A16" s="12" t="s">
@@ -978,14 +1194,30 @@
       <c r="B16" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
+      <c r="C16" s="8">
+        <v>380000</v>
+      </c>
+      <c r="D16" s="15"/>
+      <c r="E16" s="8">
+        <f t="shared" si="0"/>
+        <v>380000</v>
+      </c>
+      <c r="F16" s="8">
+        <v>304000</v>
+      </c>
+      <c r="G16" s="8">
+        <v>243200</v>
+      </c>
+      <c r="H16" s="8">
+        <v>391000</v>
+      </c>
+      <c r="I16" s="8">
+        <f t="shared" si="1"/>
+        <v>-11000</v>
+      </c>
+      <c r="J16" s="19">
+        <v>0.65</v>
+      </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A17" s="13" t="s">
@@ -994,14 +1226,32 @@
       <c r="B17" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+      <c r="C17" s="9">
+        <v>290000</v>
+      </c>
+      <c r="D17" s="16">
+        <v>28000</v>
+      </c>
+      <c r="E17" s="9">
+        <f t="shared" si="0"/>
+        <v>318000</v>
+      </c>
+      <c r="F17" s="9">
+        <v>238500</v>
+      </c>
+      <c r="G17" s="9">
+        <v>190800</v>
+      </c>
+      <c r="H17" s="9">
+        <v>325000</v>
+      </c>
+      <c r="I17" s="9">
+        <f t="shared" si="1"/>
+        <v>-7000</v>
+      </c>
+      <c r="J17" s="20">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A18" s="12" t="s">
@@ -1010,14 +1260,30 @@
       <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+      <c r="C18" s="8">
+        <v>120000</v>
+      </c>
+      <c r="D18" s="15"/>
+      <c r="E18" s="8">
+        <f t="shared" si="0"/>
+        <v>120000</v>
+      </c>
+      <c r="F18" s="8">
+        <v>84000</v>
+      </c>
+      <c r="G18" s="8">
+        <v>67200</v>
+      </c>
+      <c r="H18" s="8">
+        <v>126000</v>
+      </c>
+      <c r="I18" s="8">
+        <f t="shared" si="1"/>
+        <v>-6000</v>
+      </c>
+      <c r="J18" s="19">
+        <v>0.55000000000000004</v>
+      </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A19" s="11" t="s">
@@ -1026,14 +1292,30 @@
       <c r="B19" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
+      <c r="C19" s="6">
+        <v>680000</v>
+      </c>
+      <c r="D19" s="14"/>
+      <c r="E19" s="6">
+        <f t="shared" si="0"/>
+        <v>680000</v>
+      </c>
+      <c r="F19" s="6">
+        <v>476000</v>
+      </c>
+      <c r="G19" s="6">
+        <v>380800</v>
+      </c>
+      <c r="H19" s="6">
+        <v>695000</v>
+      </c>
+      <c r="I19" s="6">
+        <f t="shared" si="1"/>
+        <v>-15000</v>
+      </c>
+      <c r="J19" s="18">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A20" s="11" t="s">
@@ -1042,14 +1324,38 @@
       <c r="B20" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
+      <c r="C20" s="6">
+        <f>SUM(C21:C23)</f>
+        <v>7030000</v>
+      </c>
+      <c r="D20" s="14">
+        <f>SUM(D21:D23)</f>
+        <v>157000</v>
+      </c>
+      <c r="E20" s="6">
+        <f t="shared" si="0"/>
+        <v>7187000</v>
+      </c>
+      <c r="F20" s="6">
+        <f>SUM(F21:F23)</f>
+        <v>6752050</v>
+      </c>
+      <c r="G20" s="6">
+        <f>SUM(G21:G23)</f>
+        <v>5403200</v>
+      </c>
+      <c r="H20" s="6">
+        <f>SUM(H21:H23)</f>
+        <v>7484000</v>
+      </c>
+      <c r="I20" s="6">
+        <f t="shared" si="1"/>
+        <v>-297000</v>
+      </c>
+      <c r="J20" s="18">
+        <f>SUMPRODUCT(E21:E23,J21:J23)/SUM(E21:E23)</f>
+        <v>0.66268262139974954</v>
+      </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A21" s="12" t="s">
@@ -1058,14 +1364,32 @@
       <c r="B21" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
+      <c r="C21" s="8">
+        <v>3240000</v>
+      </c>
+      <c r="D21" s="15">
+        <v>95000</v>
+      </c>
+      <c r="E21" s="8">
+        <f t="shared" si="0"/>
+        <v>3335000</v>
+      </c>
+      <c r="F21" s="8">
+        <v>3168250</v>
+      </c>
+      <c r="G21" s="8">
+        <v>2534600</v>
+      </c>
+      <c r="H21" s="8">
+        <v>3480000</v>
+      </c>
+      <c r="I21" s="8">
+        <f t="shared" si="1"/>
+        <v>-145000</v>
+      </c>
+      <c r="J21" s="19">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A22" s="13" t="s">
@@ -1074,14 +1398,30 @@
       <c r="B22" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
+      <c r="C22" s="9">
+        <v>2340000</v>
+      </c>
+      <c r="D22" s="16"/>
+      <c r="E22" s="9">
+        <f t="shared" si="0"/>
+        <v>2340000</v>
+      </c>
+      <c r="F22" s="9">
+        <v>2223000</v>
+      </c>
+      <c r="G22" s="9">
+        <v>1780000</v>
+      </c>
+      <c r="H22" s="9">
+        <v>2456000</v>
+      </c>
+      <c r="I22" s="9">
+        <f t="shared" si="1"/>
+        <v>-116000</v>
+      </c>
+      <c r="J22" s="20">
+        <v>0.65</v>
+      </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A23" s="12" t="s">
@@ -1090,14 +1430,32 @@
       <c r="B23" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="C23" s="8">
+        <v>1450000</v>
+      </c>
+      <c r="D23" s="15">
+        <v>62000</v>
+      </c>
+      <c r="E23" s="8">
+        <f t="shared" si="0"/>
+        <v>1512000</v>
+      </c>
+      <c r="F23" s="8">
+        <v>1360800</v>
+      </c>
+      <c r="G23" s="8">
+        <v>1088600</v>
+      </c>
+      <c r="H23" s="8">
+        <v>1548000</v>
+      </c>
+      <c r="I23" s="8">
+        <f t="shared" si="1"/>
+        <v>-36000</v>
+      </c>
+      <c r="J23" s="19">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A24" s="11" t="s">
@@ -1106,14 +1464,30 @@
       <c r="B24" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
+      <c r="C24" s="6">
+        <v>600000</v>
+      </c>
+      <c r="D24" s="14"/>
+      <c r="E24" s="6">
+        <f t="shared" si="0"/>
+        <v>600000</v>
+      </c>
+      <c r="F24" s="6">
+        <v>360000</v>
+      </c>
+      <c r="G24" s="6">
+        <v>216000</v>
+      </c>
+      <c r="H24" s="6">
+        <v>628000</v>
+      </c>
+      <c r="I24" s="6">
+        <f t="shared" si="1"/>
+        <v>-28000</v>
+      </c>
+      <c r="J24" s="18">
+        <v>0.45</v>
+      </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A25" s="11" t="s">
@@ -1122,14 +1496,32 @@
       <c r="B25" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
+      <c r="C25" s="6">
+        <v>2800000</v>
+      </c>
+      <c r="D25" s="14">
+        <v>85000</v>
+      </c>
+      <c r="E25" s="6">
+        <f t="shared" si="0"/>
+        <v>2885000</v>
+      </c>
+      <c r="F25" s="6">
+        <v>2885000</v>
+      </c>
+      <c r="G25" s="6">
+        <v>2596500</v>
+      </c>
+      <c r="H25" s="6">
+        <v>3100000</v>
+      </c>
+      <c r="I25" s="6">
+        <f t="shared" si="1"/>
+        <v>-215000</v>
+      </c>
+      <c r="J25" s="18">
+        <v>0.65</v>
+      </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A26" s="11" t="s">
@@ -1138,27 +1530,67 @@
       <c r="B26" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
+      <c r="C26" s="6">
+        <v>1010000</v>
+      </c>
+      <c r="D26" s="14"/>
+      <c r="E26" s="6">
+        <f t="shared" si="0"/>
+        <v>1010000</v>
+      </c>
+      <c r="F26" s="6">
+        <v>0</v>
+      </c>
+      <c r="G26" s="6">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6">
+        <v>850000</v>
+      </c>
+      <c r="I26" s="6">
+        <f t="shared" si="1"/>
+        <v>160000</v>
+      </c>
+      <c r="J26" s="18">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B27" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
+      <c r="C27" s="7">
+        <f>SUM(C5,C8,C15,C19,C20,C24,C25,C26)</f>
+        <v>18000000</v>
+      </c>
+      <c r="D27" s="17">
+        <f>SUM(D5,D8,D15,D19,D20,D24,D25,D26)</f>
+        <v>315000</v>
+      </c>
+      <c r="E27" s="17">
+        <f>SUM(E5,E8,E15,E19,E20,E24,E25,E26)</f>
+        <v>18315000</v>
+      </c>
+      <c r="F27" s="7">
+        <f>SUM(F5,F8,F15,F19,F20,F24,F25,F26)</f>
+        <v>16020550</v>
+      </c>
+      <c r="G27" s="7">
+        <f>SUM(G5,G8,G15,G19,G20,G24,G25,G26)</f>
+        <v>13526650</v>
+      </c>
+      <c r="H27" s="7">
+        <f>SUM(H5,H8,H15,H19,H20,H24,H25,H26)</f>
+        <v>18719000</v>
+      </c>
+      <c r="I27" s="7">
+        <f t="shared" si="1"/>
+        <v>-404000</v>
+      </c>
+      <c r="J27" s="21">
+        <f>SUMPRODUCT(E5:E26,J5:J26)/SUM(E5:E26)</f>
+        <v>0.72216658718804638</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
add variance RAG conditional formatting to cost plan
</commit_message>
<xml_diff>
--- a/cost-plans/NHS-Acute-Hospital-Wing.xlsx
+++ b/cost-plans/NHS-Acute-Hospital-Wing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3638E78-CF86-4C36-84C9-D74999CBBF7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4AAE3D-11D2-4CE6-A5A2-1AFB08B2DA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
+    <workbookView xWindow="-28920" yWindow="2355" windowWidth="29040" windowHeight="16440" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Plan" sheetId="1" r:id="rId1"/>
@@ -347,9 +347,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -374,16 +371,76 @@
     <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="2" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFC000"/>
+      <color rgb="FFFF0000"/>
       <color rgb="FF1F3864"/>
       <color rgb="FFD9D9D9"/>
       <color rgb="FF2E5496"/>
@@ -753,35 +810,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="21"/>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -813,781 +870,781 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <f>SUM(C6:C7)</f>
         <v>800000</v>
       </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="6">
+      <c r="D5" s="13"/>
+      <c r="E5" s="5">
         <f>SUM(C5:D5)</f>
         <v>800000</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <f>SUM(F6:F7)</f>
         <v>800000</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="5">
         <f>SUM(G6:G7)</f>
         <v>720000</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="5">
         <f>SUM(H6:H7)</f>
         <v>805000</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="5">
         <f>E5-H5</f>
         <v>-5000</v>
       </c>
-      <c r="J5" s="18">
+      <c r="J5" s="17">
         <f>SUMPRODUCT(E6:E7, J6:J7)/SUM(E6:E7)</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <v>540000</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="8">
-        <f t="shared" ref="E6:F26" si="0">SUM(C6:D6)</f>
+      <c r="D6" s="14"/>
+      <c r="E6" s="7">
+        <f t="shared" ref="E6:E26" si="0">SUM(C6:D6)</f>
         <v>540000</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="7">
         <v>540000</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <v>486000</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>540000</v>
       </c>
-      <c r="I6" s="8">
+      <c r="I6" s="7">
         <f t="shared" ref="I6:I27" si="1">E6-H6</f>
         <v>0</v>
       </c>
-      <c r="J6" s="19">
+      <c r="J6" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="8">
         <v>260000</v>
       </c>
-      <c r="D7" s="16"/>
-      <c r="E7" s="9">
+      <c r="D7" s="15"/>
+      <c r="E7" s="8">
         <f t="shared" si="0"/>
         <v>260000</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="8">
         <v>260000</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="8">
         <v>234000</v>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="8">
         <v>265000</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="8">
         <f t="shared" si="1"/>
         <v>-5000</v>
       </c>
-      <c r="J7" s="20">
+      <c r="J7" s="19">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <f>SUM(C9:C14)</f>
         <v>4290000</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="13">
         <f>SUM(D9:D14)</f>
         <v>45000</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="5">
         <f t="shared" si="0"/>
         <v>4335000</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="5">
         <f>SUM(F9:F14)</f>
         <v>4121000</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="5">
         <f>SUM(G9:G14)</f>
         <v>3708950</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="5">
         <f>SUM(H9:H14)</f>
         <v>4315000</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="5">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
-      <c r="J8" s="18">
+      <c r="J8" s="17">
         <f>SUMPRODUCT(E9:E14,J9:J14)/SUM(E9:E14)</f>
         <v>0.92612456747404848</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <v>1800000</v>
       </c>
-      <c r="D9" s="15"/>
-      <c r="E9" s="8">
+      <c r="D9" s="14"/>
+      <c r="E9" s="7">
         <f t="shared" si="0"/>
         <v>1800000</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="7">
         <v>1800000</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <v>1620000</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="7">
         <v>1800000</v>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="7">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="8">
         <v>650000</v>
       </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="9">
+      <c r="D10" s="15"/>
+      <c r="E10" s="8">
         <f t="shared" si="0"/>
         <v>650000</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="8">
         <v>650000</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="8">
         <v>585000</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="8">
         <v>650000</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="8">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J10" s="20">
+      <c r="J10" s="19">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="7">
         <v>280000</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="8">
+      <c r="D11" s="14"/>
+      <c r="E11" s="7">
         <f t="shared" si="0"/>
         <v>280000</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="7">
         <v>266000</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="7">
         <v>239400</v>
       </c>
-      <c r="H11" s="8">
+      <c r="H11" s="7">
         <v>272000</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="7">
         <f t="shared" si="1"/>
         <v>8000</v>
       </c>
-      <c r="J11" s="19">
+      <c r="J11" s="18">
         <v>0.95</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>950000</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="15">
         <v>45000</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="8">
         <f t="shared" si="0"/>
         <v>995000</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="8">
         <v>895500</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="8">
         <v>806000</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="8">
         <v>1045000</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="8">
         <f t="shared" si="1"/>
         <v>-50000</v>
       </c>
-      <c r="J12" s="20">
+      <c r="J12" s="19">
         <v>0.85</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="7">
         <v>520000</v>
       </c>
-      <c r="D13" s="15"/>
-      <c r="E13" s="8">
+      <c r="D13" s="14"/>
+      <c r="E13" s="7">
         <f t="shared" si="0"/>
         <v>520000</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="7">
         <v>442000</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="7">
         <v>397800</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H13" s="7">
         <v>476000</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="7">
         <f t="shared" si="1"/>
         <v>44000</v>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="18">
         <v>0.75</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>90000</v>
       </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="9">
+      <c r="D14" s="15"/>
+      <c r="E14" s="8">
         <f t="shared" si="0"/>
         <v>90000</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="8">
         <v>67500</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="8">
         <v>60750</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="8">
         <v>72000</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="8">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
-      <c r="J14" s="20">
+      <c r="J14" s="19">
         <v>0.7</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="5">
         <f>SUM(C16:C18)</f>
         <v>790000</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="13">
         <f>SUM(D16:D18)</f>
         <v>28000</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="5">
         <f t="shared" si="0"/>
         <v>818000</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="5">
         <f>SUM(F16:F18)</f>
         <v>626500</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="5">
         <f>SUM(G16:G18)</f>
         <v>501200</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H15" s="5">
         <f>SUM(H16:H18)</f>
         <v>842000</v>
       </c>
-      <c r="I15" s="6">
+      <c r="I15" s="5">
         <f t="shared" si="1"/>
         <v>-24000</v>
       </c>
-      <c r="J15" s="18">
+      <c r="J15" s="17">
         <f>SUMPRODUCT(E16:E18,J16:J18)/SUM(E16:E18)</f>
         <v>0.61589242053789728</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="7">
         <v>380000</v>
       </c>
-      <c r="D16" s="15"/>
-      <c r="E16" s="8">
+      <c r="D16" s="14"/>
+      <c r="E16" s="7">
         <f t="shared" si="0"/>
         <v>380000</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="7">
         <v>304000</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="7">
         <v>243200</v>
       </c>
-      <c r="H16" s="8">
+      <c r="H16" s="7">
         <v>391000</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="7">
         <f t="shared" si="1"/>
         <v>-11000</v>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="18">
         <v>0.65</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="9">
+      <c r="C17" s="8">
         <v>290000</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="15">
         <v>28000</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="8">
         <f t="shared" si="0"/>
         <v>318000</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="8">
         <v>238500</v>
       </c>
-      <c r="G17" s="9">
+      <c r="G17" s="8">
         <v>190800</v>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="8">
         <v>325000</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="8">
         <f t="shared" si="1"/>
         <v>-7000</v>
       </c>
-      <c r="J17" s="20">
+      <c r="J17" s="19">
         <v>0.6</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="7">
         <v>120000</v>
       </c>
-      <c r="D18" s="15"/>
-      <c r="E18" s="8">
+      <c r="D18" s="14"/>
+      <c r="E18" s="7">
         <f t="shared" si="0"/>
         <v>120000</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="7">
         <v>84000</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="7">
         <v>67200</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="7">
         <v>126000</v>
       </c>
-      <c r="I18" s="8">
+      <c r="I18" s="7">
         <f t="shared" si="1"/>
         <v>-6000</v>
       </c>
-      <c r="J18" s="19">
+      <c r="J18" s="18">
         <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="5">
         <v>680000</v>
       </c>
-      <c r="D19" s="14"/>
-      <c r="E19" s="6">
+      <c r="D19" s="13"/>
+      <c r="E19" s="5">
         <f t="shared" si="0"/>
         <v>680000</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="5">
         <v>476000</v>
       </c>
-      <c r="G19" s="6">
+      <c r="G19" s="5">
         <v>380800</v>
       </c>
-      <c r="H19" s="6">
+      <c r="H19" s="5">
         <v>695000</v>
       </c>
-      <c r="I19" s="6">
+      <c r="I19" s="5">
         <f t="shared" si="1"/>
         <v>-15000</v>
       </c>
-      <c r="J19" s="18">
+      <c r="J19" s="17">
         <v>0.6</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C20" s="6">
+      <c r="C20" s="5">
         <f>SUM(C21:C23)</f>
         <v>7030000</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="13">
         <f>SUM(D21:D23)</f>
         <v>157000</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="5">
         <f t="shared" si="0"/>
         <v>7187000</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="5">
         <f>SUM(F21:F23)</f>
         <v>6752050</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="5">
         <f>SUM(G21:G23)</f>
         <v>5403200</v>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="5">
         <f>SUM(H21:H23)</f>
         <v>7484000</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="5">
         <f t="shared" si="1"/>
         <v>-297000</v>
       </c>
-      <c r="J20" s="18">
+      <c r="J20" s="17">
         <f>SUMPRODUCT(E21:E23,J21:J23)/SUM(E21:E23)</f>
         <v>0.66268262139974954</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="7">
         <v>3240000</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="14">
         <v>95000</v>
       </c>
-      <c r="E21" s="8">
+      <c r="E21" s="7">
         <f t="shared" si="0"/>
         <v>3335000</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F21" s="7">
         <v>3168250</v>
       </c>
-      <c r="G21" s="8">
+      <c r="G21" s="7">
         <v>2534600</v>
       </c>
-      <c r="H21" s="8">
+      <c r="H21" s="7">
         <v>3480000</v>
       </c>
-      <c r="I21" s="8">
+      <c r="I21" s="7">
         <f t="shared" si="1"/>
         <v>-145000</v>
       </c>
-      <c r="J21" s="19">
+      <c r="J21" s="18">
         <v>0.7</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C22" s="9">
+      <c r="C22" s="8">
         <v>2340000</v>
       </c>
-      <c r="D22" s="16"/>
-      <c r="E22" s="9">
+      <c r="D22" s="15"/>
+      <c r="E22" s="8">
         <f t="shared" si="0"/>
         <v>2340000</v>
       </c>
-      <c r="F22" s="9">
+      <c r="F22" s="8">
         <v>2223000</v>
       </c>
-      <c r="G22" s="9">
+      <c r="G22" s="8">
         <v>1780000</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="8">
         <v>2456000</v>
       </c>
-      <c r="I22" s="9">
+      <c r="I22" s="8">
         <f t="shared" si="1"/>
         <v>-116000</v>
       </c>
-      <c r="J22" s="20">
+      <c r="J22" s="19">
         <v>0.65</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="7">
         <v>1450000</v>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="14">
         <v>62000</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E23" s="7">
         <f t="shared" si="0"/>
         <v>1512000</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F23" s="7">
         <v>1360800</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="7">
         <v>1088600</v>
       </c>
-      <c r="H23" s="8">
+      <c r="H23" s="7">
         <v>1548000</v>
       </c>
-      <c r="I23" s="8">
+      <c r="I23" s="7">
         <f t="shared" si="1"/>
         <v>-36000</v>
       </c>
-      <c r="J23" s="19">
+      <c r="J23" s="18">
         <v>0.6</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="5">
         <v>600000</v>
       </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="6">
+      <c r="D24" s="13"/>
+      <c r="E24" s="5">
         <f t="shared" si="0"/>
         <v>600000</v>
       </c>
-      <c r="F24" s="6">
+      <c r="F24" s="5">
         <v>360000</v>
       </c>
-      <c r="G24" s="6">
+      <c r="G24" s="5">
         <v>216000</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="5">
         <v>628000</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="5">
         <f t="shared" si="1"/>
         <v>-28000</v>
       </c>
-      <c r="J24" s="18">
+      <c r="J24" s="17">
         <v>0.45</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="5">
         <v>2800000</v>
       </c>
-      <c r="D25" s="14">
+      <c r="D25" s="13">
         <v>85000</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="5">
         <f t="shared" si="0"/>
         <v>2885000</v>
       </c>
-      <c r="F25" s="6">
+      <c r="F25" s="5">
         <v>2885000</v>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="5">
         <v>2596500</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="5">
         <v>3100000</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="5">
         <f t="shared" si="1"/>
         <v>-215000</v>
       </c>
-      <c r="J25" s="18">
+      <c r="J25" s="17">
         <v>0.65</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C26" s="6">
+      <c r="C26" s="5">
         <v>1010000</v>
       </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="6">
+      <c r="D26" s="13"/>
+      <c r="E26" s="5">
         <f t="shared" si="0"/>
         <v>1010000</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="5">
         <v>0</v>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="5">
         <v>0</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="5">
         <v>850000</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="5">
         <f t="shared" si="1"/>
         <v>160000</v>
       </c>
-      <c r="J26" s="18">
+      <c r="J26" s="17">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="7">
-        <f>SUM(C5,C8,C15,C19,C20,C24,C25,C26)</f>
+      <c r="C27" s="6">
+        <f t="shared" ref="C27:H27" si="2">SUM(C5,C8,C15,C19,C20,C24,C25,C26)</f>
         <v>18000000</v>
       </c>
-      <c r="D27" s="17">
-        <f>SUM(D5,D8,D15,D19,D20,D24,D25,D26)</f>
+      <c r="D27" s="16">
+        <f t="shared" si="2"/>
         <v>315000</v>
       </c>
-      <c r="E27" s="17">
-        <f>SUM(E5,E8,E15,E19,E20,E24,E25,E26)</f>
+      <c r="E27" s="16">
+        <f t="shared" si="2"/>
         <v>18315000</v>
       </c>
-      <c r="F27" s="7">
-        <f>SUM(F5,F8,F15,F19,F20,F24,F25,F26)</f>
+      <c r="F27" s="6">
+        <f t="shared" si="2"/>
         <v>16020550</v>
       </c>
-      <c r="G27" s="7">
-        <f>SUM(G5,G8,G15,G19,G20,G24,G25,G26)</f>
+      <c r="G27" s="6">
+        <f t="shared" si="2"/>
         <v>13526650</v>
       </c>
-      <c r="H27" s="7">
-        <f>SUM(H5,H8,H15,H19,H20,H24,H25,H26)</f>
+      <c r="H27" s="6">
+        <f t="shared" si="2"/>
         <v>18719000</v>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="6">
         <f t="shared" si="1"/>
         <v>-404000</v>
       </c>
-      <c r="J27" s="21">
+      <c r="J27" s="20">
         <f>SUMPRODUCT(E5:E26,J5:J26)/SUM(E5:E26)</f>
         <v>0.72216658718804638</v>
       </c>
@@ -1597,6 +1654,14 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
+  <conditionalFormatting sqref="I5:I27">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>AND(I5&lt;0, I5&gt;=-E5*0.02)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A5:A26" numberStoredAsText="1"/>

</xml_diff>

<commit_message>
complete NHS hospital CVR tab with formatting and chart
</commit_message>
<xml_diff>
--- a/cost-plans/NHS-Acute-Hospital-Wing.xlsx
+++ b/cost-plans/NHS-Acute-Hospital-Wing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4AAE3D-11D2-4CE6-A5A2-1AFB08B2DA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0344444F-A93B-4477-A8D8-57AC927EDF56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2355" windowWidth="29040" windowHeight="16440" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Plan" sheetId="1" r:id="rId1"/>
@@ -257,7 +257,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -281,6 +281,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -339,7 +347,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -374,13 +382,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
     <dxf>
       <font>
         <color theme="0"/>
@@ -409,14 +421,22 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FF70AD47"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
         <color theme="0"/>
       </font>
       <fill>
@@ -439,6 +459,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF70AD47"/>
       <color rgb="FFFFC000"/>
       <color rgb="FFFF0000"/>
       <color rgb="FF1F3864"/>
@@ -797,7 +818,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B8CA9C0-9C58-4F75-869D-8D1A35F325AC}">
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.6" outlineLevelRow="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="12.69140625" style="4" customWidth="1"/>
     <col min="2" max="2" width="35.69140625" customWidth="1"/>
@@ -897,7 +918,7 @@
         <f>SUM(H6:H7)</f>
         <v>805000</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="22">
         <f>E5-H5</f>
         <v>-5000</v>
       </c>
@@ -906,7 +927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A6" s="11" t="s">
         <v>26</v>
       </c>
@@ -930,7 +951,7 @@
       <c r="H6" s="7">
         <v>540000</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="23">
         <f t="shared" ref="I6:I27" si="1">E6-H6</f>
         <v>0</v>
       </c>
@@ -938,7 +959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A7" s="12" t="s">
         <v>27</v>
       </c>
@@ -962,7 +983,7 @@
       <c r="H7" s="8">
         <v>265000</v>
       </c>
-      <c r="I7" s="8">
+      <c r="I7" s="24">
         <f t="shared" si="1"/>
         <v>-5000</v>
       </c>
@@ -1001,7 +1022,7 @@
         <f>SUM(H9:H14)</f>
         <v>4315000</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="22">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
@@ -1010,7 +1031,7 @@
         <v>0.92612456747404848</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A9" s="11" t="s">
         <v>29</v>
       </c>
@@ -1034,7 +1055,7 @@
       <c r="H9" s="7">
         <v>1800000</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="23">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1042,7 +1063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A10" s="12" t="s">
         <v>30</v>
       </c>
@@ -1066,7 +1087,7 @@
       <c r="H10" s="8">
         <v>650000</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1074,7 +1095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A11" s="11" t="s">
         <v>31</v>
       </c>
@@ -1098,7 +1119,7 @@
       <c r="H11" s="7">
         <v>272000</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="23">
         <f t="shared" si="1"/>
         <v>8000</v>
       </c>
@@ -1106,7 +1127,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A12" s="12" t="s">
         <v>32</v>
       </c>
@@ -1132,7 +1153,7 @@
       <c r="H12" s="8">
         <v>1045000</v>
       </c>
-      <c r="I12" s="8">
+      <c r="I12" s="24">
         <f t="shared" si="1"/>
         <v>-50000</v>
       </c>
@@ -1140,7 +1161,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A13" s="11" t="s">
         <v>33</v>
       </c>
@@ -1164,7 +1185,7 @@
       <c r="H13" s="7">
         <v>476000</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="23">
         <f t="shared" si="1"/>
         <v>44000</v>
       </c>
@@ -1172,7 +1193,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A14" s="12" t="s">
         <v>34</v>
       </c>
@@ -1196,7 +1217,7 @@
       <c r="H14" s="8">
         <v>72000</v>
       </c>
-      <c r="I14" s="8">
+      <c r="I14" s="24">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
@@ -1235,7 +1256,7 @@
         <f>SUM(H16:H18)</f>
         <v>842000</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="22">
         <f t="shared" si="1"/>
         <v>-24000</v>
       </c>
@@ -1244,7 +1265,7 @@
         <v>0.61589242053789728</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A16" s="11" t="s">
         <v>36</v>
       </c>
@@ -1268,7 +1289,7 @@
       <c r="H16" s="7">
         <v>391000</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="23">
         <f t="shared" si="1"/>
         <v>-11000</v>
       </c>
@@ -1276,7 +1297,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A17" s="12" t="s">
         <v>37</v>
       </c>
@@ -1302,7 +1323,7 @@
       <c r="H17" s="8">
         <v>325000</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="24">
         <f t="shared" si="1"/>
         <v>-7000</v>
       </c>
@@ -1310,7 +1331,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A18" s="11" t="s">
         <v>38</v>
       </c>
@@ -1334,7 +1355,7 @@
       <c r="H18" s="7">
         <v>126000</v>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="23">
         <f t="shared" si="1"/>
         <v>-6000</v>
       </c>
@@ -1366,7 +1387,7 @@
       <c r="H19" s="5">
         <v>695000</v>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="22">
         <f t="shared" si="1"/>
         <v>-15000</v>
       </c>
@@ -1405,7 +1426,7 @@
         <f>SUM(H21:H23)</f>
         <v>7484000</v>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="22">
         <f t="shared" si="1"/>
         <v>-297000</v>
       </c>
@@ -1414,7 +1435,7 @@
         <v>0.66268262139974954</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A21" s="11" t="s">
         <v>41</v>
       </c>
@@ -1440,7 +1461,7 @@
       <c r="H21" s="7">
         <v>3480000</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="23">
         <f t="shared" si="1"/>
         <v>-145000</v>
       </c>
@@ -1448,7 +1469,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A22" s="12" t="s">
         <v>42</v>
       </c>
@@ -1472,7 +1493,7 @@
       <c r="H22" s="8">
         <v>2456000</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="24">
         <f t="shared" si="1"/>
         <v>-116000</v>
       </c>
@@ -1480,7 +1501,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A23" s="11" t="s">
         <v>43</v>
       </c>
@@ -1506,7 +1527,7 @@
       <c r="H23" s="7">
         <v>1548000</v>
       </c>
-      <c r="I23" s="7">
+      <c r="I23" s="23">
         <f t="shared" si="1"/>
         <v>-36000</v>
       </c>
@@ -1538,7 +1559,7 @@
       <c r="H24" s="5">
         <v>628000</v>
       </c>
-      <c r="I24" s="5">
+      <c r="I24" s="22">
         <f t="shared" si="1"/>
         <v>-28000</v>
       </c>
@@ -1572,7 +1593,7 @@
       <c r="H25" s="5">
         <v>3100000</v>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="22">
         <f t="shared" si="1"/>
         <v>-215000</v>
       </c>
@@ -1604,7 +1625,7 @@
       <c r="H26" s="5">
         <v>850000</v>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="22">
         <f t="shared" si="1"/>
         <v>160000</v>
       </c>
@@ -1640,7 +1661,7 @@
         <f t="shared" si="2"/>
         <v>18719000</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="25">
         <f t="shared" si="1"/>
         <v>-404000</v>
       </c>
@@ -1655,11 +1676,14 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:I27">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>AND(I5&lt;0, I5&gt;=-E5*0.02)</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add project build guide PDF
</commit_message>
<xml_diff>
--- a/cost-plans/NHS-Acute-Hospital-Wing.xlsx
+++ b/cost-plans/NHS-Acute-Hospital-Wing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0344444F-A93B-4477-A8D8-57AC927EDF56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE4E5CE-50D6-4F75-8130-EB78E9A3B4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="1" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Plan" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="78">
   <si>
     <t>Project Name</t>
   </si>
@@ -88,9 +88,6 @@
     <t>NHS Acute Hospital Wing — Elemental Cost Plan</t>
   </si>
   <si>
-    <t>Meridian Cost Consultants | Report Date: [we'll make this dynamic later]</t>
-  </si>
-  <si>
     <t>Element Ref</t>
   </si>
   <si>
@@ -251,13 +248,45 @@
   </si>
   <si>
     <t>Total Project Cost</t>
+  </si>
+  <si>
+    <t>NHS Acute Hospital Wing — Cost Value Reconciliation</t>
+  </si>
+  <si>
+    <t>Meridian Cost Consultants | Reporting Period: September 2024</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Cumulative Value (£)</t>
+  </si>
+  <si>
+    <t>Cumulative Cost (£)</t>
+  </si>
+  <si>
+    <t>Gross Margin (£)</t>
+  </si>
+  <si>
+    <t>Margin %</t>
+  </si>
+  <si>
+    <t>CPI</t>
+  </si>
+  <si>
+    <t>EAC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -291,6 +320,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -333,7 +370,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -341,13 +378,100 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -379,32 +503,73 @@
     <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="2" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="17" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="5" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="38" fontId="0" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="38" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="38" fontId="0" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
+    <cellStyle name="Comma" xfId="3" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
         <color theme="0"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF70AD47"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color theme="0"/>
       </font>
       <fill>
@@ -445,26 +610,16 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FF70AD47"/>
-      <color rgb="FFFFC000"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF2E5496"/>
       <color rgb="FF1F3864"/>
       <color rgb="FFD9D9D9"/>
-      <color rgb="FF2E5496"/>
+      <color rgb="FF70AD47"/>
+      <color rgb="FFFF0000"/>
+      <color rgb="FFFFC000"/>
     </mruColors>
   </colors>
   <extLst>
@@ -476,6 +631,1224 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Cumulative Value vs Cost — NHS Acute Hospital Wing</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>CVR!$B$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Cumulative Value (£)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="1F3864"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="1F3864"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-1.6969695761016267E-2"/>
+                  <c:y val="7.1065502058144367E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-8567-424D-8F78-650AFDB2B1C9}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:numFmt formatCode="&quot;£&quot;#,##0.0,,&quot;M&quot;" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>CVR!$A$5:$A$10</c:f>
+              <c:numCache>
+                <c:formatCode>mmm\-yy</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>45383</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45413</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45474</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45505</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>45536</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>CVR!$B$5:$B$10</c:f>
+              <c:numCache>
+                <c:formatCode>_-* #,##0_-;\-* #,##0_-;_-* "-"??_-;_-@_-</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>850000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1920000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3450000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5280000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8640000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>11850000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8567-424D-8F78-650AFDB2B1C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>CVR!$C$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Cumulative Cost (£)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-8.2400114740059094E-2"/>
+                  <c:y val="-6.0082038925462183E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-8567-424D-8F78-650AFDB2B1C9}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:numFmt formatCode="&quot;£&quot;#,##0.0,,&quot;M&quot;" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>CVR!$A$5:$A$10</c:f>
+              <c:numCache>
+                <c:formatCode>mmm\-yy</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>45383</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>45413</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45444</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>45474</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45505</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>45536</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>CVR!$C$5:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>_-* #,##0_-;\-* #,##0_-;_-* "-"??_-;_-@_-</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>820000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1850000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3350000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5180000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8750000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>12254650</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-8567-424D-8F78-650AFDB2B1C9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1240057632"/>
+        <c:axId val="1240059072"/>
+      </c:lineChart>
+      <c:dateAx>
+        <c:axId val="1240057632"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="mmm\-yy" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1240059072"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblOffset val="100"/>
+        <c:baseTimeUnit val="months"/>
+      </c:dateAx>
+      <c:valAx>
+        <c:axId val="1240059072"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="&quot;£&quot;#,##0.0,,&quot;M&quot;" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1240057632"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2720</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1159328</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>174172</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3FE3656-B091-E91D-957A-6A1A3B01089E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -830,61 +2203,62 @@
     <col min="10" max="10" width="14.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:10" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+    </row>
+    <row r="2" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="41" t="str">
+        <f ca="1">"Meridian Cost Consultants | Report Date: "&amp;TEXT(TODAY(),"DD MMMM YYYY")</f>
+        <v>Meridian Cost Consultants | Report Date: 13 May 2026</v>
+      </c>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>12</v>
@@ -892,10 +2266,10 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A5" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C5" s="5">
         <f>SUM(C6:C7)</f>
@@ -918,7 +2292,7 @@
         <f>SUM(H6:H7)</f>
         <v>805000</v>
       </c>
-      <c r="I5" s="22">
+      <c r="I5" s="21">
         <f>E5-H5</f>
         <v>-5000</v>
       </c>
@@ -929,10 +2303,10 @@
     </row>
     <row r="6" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A6" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C6" s="7">
         <v>540000</v>
@@ -951,7 +2325,7 @@
       <c r="H6" s="7">
         <v>540000</v>
       </c>
-      <c r="I6" s="23">
+      <c r="I6" s="22">
         <f t="shared" ref="I6:I27" si="1">E6-H6</f>
         <v>0</v>
       </c>
@@ -961,10 +2335,10 @@
     </row>
     <row r="7" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A7" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C7" s="8">
         <v>260000</v>
@@ -983,7 +2357,7 @@
       <c r="H7" s="8">
         <v>265000</v>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="23">
         <f t="shared" si="1"/>
         <v>-5000</v>
       </c>
@@ -993,10 +2367,10 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A8" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C8" s="5">
         <f>SUM(C9:C14)</f>
@@ -1022,7 +2396,7 @@
         <f>SUM(H9:H14)</f>
         <v>4315000</v>
       </c>
-      <c r="I8" s="22">
+      <c r="I8" s="21">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
@@ -1033,10 +2407,10 @@
     </row>
     <row r="9" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A9" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" s="7">
         <v>1800000</v>
@@ -1055,7 +2429,7 @@
       <c r="H9" s="7">
         <v>1800000</v>
       </c>
-      <c r="I9" s="23">
+      <c r="I9" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1065,10 +2439,10 @@
     </row>
     <row r="10" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A10" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C10" s="8">
         <v>650000</v>
@@ -1087,7 +2461,7 @@
       <c r="H10" s="8">
         <v>650000</v>
       </c>
-      <c r="I10" s="24">
+      <c r="I10" s="23">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1097,10 +2471,10 @@
     </row>
     <row r="11" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A11" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C11" s="7">
         <v>280000</v>
@@ -1119,7 +2493,7 @@
       <c r="H11" s="7">
         <v>272000</v>
       </c>
-      <c r="I11" s="23">
+      <c r="I11" s="22">
         <f t="shared" si="1"/>
         <v>8000</v>
       </c>
@@ -1129,10 +2503,10 @@
     </row>
     <row r="12" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A12" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C12" s="8">
         <v>950000</v>
@@ -1153,7 +2527,7 @@
       <c r="H12" s="8">
         <v>1045000</v>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="23">
         <f t="shared" si="1"/>
         <v>-50000</v>
       </c>
@@ -1163,10 +2537,10 @@
     </row>
     <row r="13" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A13" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C13" s="7">
         <v>520000</v>
@@ -1185,7 +2559,7 @@
       <c r="H13" s="7">
         <v>476000</v>
       </c>
-      <c r="I13" s="23">
+      <c r="I13" s="22">
         <f t="shared" si="1"/>
         <v>44000</v>
       </c>
@@ -1195,10 +2569,10 @@
     </row>
     <row r="14" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A14" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C14" s="8">
         <v>90000</v>
@@ -1217,7 +2591,7 @@
       <c r="H14" s="8">
         <v>72000</v>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="23">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
@@ -1227,10 +2601,10 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A15" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C15" s="5">
         <f>SUM(C16:C18)</f>
@@ -1256,7 +2630,7 @@
         <f>SUM(H16:H18)</f>
         <v>842000</v>
       </c>
-      <c r="I15" s="22">
+      <c r="I15" s="21">
         <f t="shared" si="1"/>
         <v>-24000</v>
       </c>
@@ -1267,10 +2641,10 @@
     </row>
     <row r="16" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A16" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C16" s="7">
         <v>380000</v>
@@ -1289,7 +2663,7 @@
       <c r="H16" s="7">
         <v>391000</v>
       </c>
-      <c r="I16" s="23">
+      <c r="I16" s="22">
         <f t="shared" si="1"/>
         <v>-11000</v>
       </c>
@@ -1299,10 +2673,10 @@
     </row>
     <row r="17" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A17" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C17" s="8">
         <v>290000</v>
@@ -1323,7 +2697,7 @@
       <c r="H17" s="8">
         <v>325000</v>
       </c>
-      <c r="I17" s="24">
+      <c r="I17" s="23">
         <f t="shared" si="1"/>
         <v>-7000</v>
       </c>
@@ -1333,10 +2707,10 @@
     </row>
     <row r="18" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A18" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C18" s="7">
         <v>120000</v>
@@ -1355,7 +2729,7 @@
       <c r="H18" s="7">
         <v>126000</v>
       </c>
-      <c r="I18" s="23">
+      <c r="I18" s="22">
         <f t="shared" si="1"/>
         <v>-6000</v>
       </c>
@@ -1365,10 +2739,10 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A19" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C19" s="5">
         <v>680000</v>
@@ -1387,7 +2761,7 @@
       <c r="H19" s="5">
         <v>695000</v>
       </c>
-      <c r="I19" s="22">
+      <c r="I19" s="21">
         <f t="shared" si="1"/>
         <v>-15000</v>
       </c>
@@ -1397,10 +2771,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A20" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C20" s="5">
         <f>SUM(C21:C23)</f>
@@ -1426,7 +2800,7 @@
         <f>SUM(H21:H23)</f>
         <v>7484000</v>
       </c>
-      <c r="I20" s="22">
+      <c r="I20" s="21">
         <f t="shared" si="1"/>
         <v>-297000</v>
       </c>
@@ -1437,10 +2811,10 @@
     </row>
     <row r="21" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A21" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C21" s="7">
         <v>3240000</v>
@@ -1461,7 +2835,7 @@
       <c r="H21" s="7">
         <v>3480000</v>
       </c>
-      <c r="I21" s="23">
+      <c r="I21" s="22">
         <f t="shared" si="1"/>
         <v>-145000</v>
       </c>
@@ -1471,10 +2845,10 @@
     </row>
     <row r="22" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A22" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C22" s="8">
         <v>2340000</v>
@@ -1493,7 +2867,7 @@
       <c r="H22" s="8">
         <v>2456000</v>
       </c>
-      <c r="I22" s="24">
+      <c r="I22" s="23">
         <f t="shared" si="1"/>
         <v>-116000</v>
       </c>
@@ -1503,10 +2877,10 @@
     </row>
     <row r="23" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A23" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C23" s="7">
         <v>1450000</v>
@@ -1527,7 +2901,7 @@
       <c r="H23" s="7">
         <v>1548000</v>
       </c>
-      <c r="I23" s="23">
+      <c r="I23" s="22">
         <f t="shared" si="1"/>
         <v>-36000</v>
       </c>
@@ -1537,10 +2911,10 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A24" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C24" s="5">
         <v>600000</v>
@@ -1559,7 +2933,7 @@
       <c r="H24" s="5">
         <v>628000</v>
       </c>
-      <c r="I24" s="22">
+      <c r="I24" s="21">
         <f t="shared" si="1"/>
         <v>-28000</v>
       </c>
@@ -1569,10 +2943,10 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A25" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C25" s="5">
         <v>2800000</v>
@@ -1593,7 +2967,7 @@
       <c r="H25" s="5">
         <v>3100000</v>
       </c>
-      <c r="I25" s="22">
+      <c r="I25" s="21">
         <f t="shared" si="1"/>
         <v>-215000</v>
       </c>
@@ -1603,10 +2977,10 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A26" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C26" s="5">
         <v>1010000</v>
@@ -1625,7 +2999,7 @@
       <c r="H26" s="5">
         <v>850000</v>
       </c>
-      <c r="I26" s="22">
+      <c r="I26" s="21">
         <f t="shared" si="1"/>
         <v>160000</v>
       </c>
@@ -1635,7 +3009,7 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.4">
       <c r="B27" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C27" s="6">
         <f t="shared" ref="C27:H27" si="2">SUM(C5,C8,C15,C19,C20,C24,C25,C26)</f>
@@ -1661,7 +3035,7 @@
         <f t="shared" si="2"/>
         <v>18719000</v>
       </c>
-      <c r="I27" s="25">
+      <c r="I27" s="24">
         <f t="shared" si="1"/>
         <v>-404000</v>
       </c>
@@ -1676,13 +3050,13 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:I27">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>AND(I5&lt;0, I5&gt;=-E5*0.02)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1695,10 +3069,248 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32E7EEEB-5485-4D53-B51F-28DE04337FA4}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G1048576"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18.69140625" customWidth="1"/>
+    <col min="2" max="4" width="22.69140625" customWidth="1"/>
+    <col min="5" max="5" width="14.69140625" customWidth="1"/>
+    <col min="6" max="6" width="10.69140625" customWidth="1"/>
+    <col min="7" max="7" width="16.69140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+    </row>
+    <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="41" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="42" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="43" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="43" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="43" t="s">
+        <v>76</v>
+      </c>
+      <c r="G4" s="44" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A5" s="25">
+        <v>45383</v>
+      </c>
+      <c r="B5" s="26">
+        <v>850000</v>
+      </c>
+      <c r="C5" s="26">
+        <v>820000</v>
+      </c>
+      <c r="D5" s="45">
+        <f>B5-C5</f>
+        <v>30000</v>
+      </c>
+      <c r="E5" s="27">
+        <f>D5/B5</f>
+        <v>3.5294117647058823E-2</v>
+      </c>
+      <c r="F5" s="28">
+        <f>B5/C5</f>
+        <v>1.0365853658536586</v>
+      </c>
+      <c r="G5" s="29">
+        <f>18315000/F5</f>
+        <v>17668588.235294119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A6" s="30">
+        <v>45413</v>
+      </c>
+      <c r="B6" s="31">
+        <v>1920000</v>
+      </c>
+      <c r="C6" s="31">
+        <v>1850000</v>
+      </c>
+      <c r="D6" s="46">
+        <f t="shared" ref="D6:D10" si="0">B6-C6</f>
+        <v>70000</v>
+      </c>
+      <c r="E6" s="32">
+        <f t="shared" ref="E6:E10" si="1">D6/B6</f>
+        <v>3.6458333333333336E-2</v>
+      </c>
+      <c r="F6" s="33">
+        <f t="shared" ref="F6:F10" si="2">B6/C6</f>
+        <v>1.0378378378378379</v>
+      </c>
+      <c r="G6" s="34">
+        <f t="shared" ref="G6:G10" si="3">18315000/F6</f>
+        <v>17647265.625</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A7" s="25">
+        <v>45444</v>
+      </c>
+      <c r="B7" s="26">
+        <v>3450000</v>
+      </c>
+      <c r="C7" s="26">
+        <v>3350000</v>
+      </c>
+      <c r="D7" s="45">
+        <f t="shared" si="0"/>
+        <v>100000</v>
+      </c>
+      <c r="E7" s="27">
+        <f t="shared" si="1"/>
+        <v>2.8985507246376812E-2</v>
+      </c>
+      <c r="F7" s="28">
+        <f t="shared" si="2"/>
+        <v>1.0298507462686568</v>
+      </c>
+      <c r="G7" s="29">
+        <f t="shared" si="3"/>
+        <v>17784130.434782606</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A8" s="30">
+        <v>45474</v>
+      </c>
+      <c r="B8" s="31">
+        <v>5280000</v>
+      </c>
+      <c r="C8" s="31">
+        <v>5180000</v>
+      </c>
+      <c r="D8" s="46">
+        <f t="shared" si="0"/>
+        <v>100000</v>
+      </c>
+      <c r="E8" s="32">
+        <f t="shared" si="1"/>
+        <v>1.893939393939394E-2</v>
+      </c>
+      <c r="F8" s="33">
+        <f t="shared" si="2"/>
+        <v>1.0193050193050193</v>
+      </c>
+      <c r="G8" s="34">
+        <f t="shared" si="3"/>
+        <v>17968125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A9" s="25">
+        <v>45505</v>
+      </c>
+      <c r="B9" s="26">
+        <v>8640000</v>
+      </c>
+      <c r="C9" s="26">
+        <v>8750000</v>
+      </c>
+      <c r="D9" s="45">
+        <f t="shared" si="0"/>
+        <v>-110000</v>
+      </c>
+      <c r="E9" s="27">
+        <f t="shared" si="1"/>
+        <v>-1.2731481481481481E-2</v>
+      </c>
+      <c r="F9" s="28">
+        <f t="shared" si="2"/>
+        <v>0.98742857142857143</v>
+      </c>
+      <c r="G9" s="29">
+        <f t="shared" si="3"/>
+        <v>18548177.083333332</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A10" s="35">
+        <v>45536</v>
+      </c>
+      <c r="B10" s="36">
+        <v>11850000</v>
+      </c>
+      <c r="C10" s="36">
+        <v>12254650</v>
+      </c>
+      <c r="D10" s="47">
+        <f t="shared" si="0"/>
+        <v>-404650</v>
+      </c>
+      <c r="E10" s="37">
+        <f t="shared" si="1"/>
+        <v>-3.4147679324894514E-2</v>
+      </c>
+      <c r="F10" s="38">
+        <f t="shared" si="2"/>
+        <v>0.96697988110635558</v>
+      </c>
+      <c r="G10" s="39">
+        <f t="shared" si="3"/>
+        <v>18940414.746835444</v>
+      </c>
+    </row>
+    <row r="1048576" spans="2:3" x14ac:dyDescent="0.4">
+      <c r="B1048576">
+        <f>SUM(B1:B1048575)</f>
+        <v>31990000</v>
+      </c>
+      <c r="C1048576">
+        <f>SUM(C1:C1048575)</f>
+        <v>32204650</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D5:D10">
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>D5&lt;0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>D5&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
add Urban Highway Improvement Scheme cost plan and CVR
</commit_message>
<xml_diff>
--- a/cost-plans/NHS-Acute-Hospital-Wing.xlsx
+++ b/cost-plans/NHS-Acute-Hospital-Wing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE4E5CE-50D6-4F75-8130-EB78E9A3B4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C802EC-DCA2-414A-97D1-74503BD634BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="1" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="2" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Plan" sheetId="1" r:id="rId1"/>
@@ -281,12 +281,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="171" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="174" formatCode="&quot;£&quot;#,##0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -328,6 +329,12 @@
       <b/>
       <sz val="14"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -471,10 +478,8 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -534,6 +539,23 @@
     <xf numFmtId="38" fontId="0" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="38" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="38" fontId="0" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="174" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
@@ -541,19 +563,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <font>
         <b/>
@@ -614,9 +624,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFD9D9D9"/>
       <color rgb="FF2E5496"/>
       <color rgb="FF1F3864"/>
-      <color rgb="FFD9D9D9"/>
       <color rgb="FF70AD47"/>
       <color rgb="FFFF0000"/>
       <color rgb="FFFFC000"/>
@@ -2193,7 +2203,7 @@
   <dimension ref="A1:J27"/>
   <sheetFormatPr defaultRowHeight="14.6" outlineLevelRow="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="12.69140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="12.69140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="35.69140625" customWidth="1"/>
     <col min="3" max="3" width="16.69140625" customWidth="1"/>
     <col min="4" max="4" width="20.69140625" customWidth="1"/>
@@ -2204,842 +2214,842 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
     </row>
     <row r="2" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="41" t="str">
+      <c r="A2" s="39" t="str">
         <f ca="1">"Meridian Cost Consultants | Report Date: "&amp;TEXT(TODAY(),"DD MMMM YYYY")</f>
         <v>Meridian Cost Consultants | Report Date: 13 May 2026</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="I2" s="41"/>
-      <c r="J2" s="41"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="3">
         <f>SUM(C6:C7)</f>
         <v>800000</v>
       </c>
-      <c r="D5" s="13"/>
-      <c r="E5" s="5">
+      <c r="D5" s="11"/>
+      <c r="E5" s="3">
         <f>SUM(C5:D5)</f>
         <v>800000</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="3">
         <f>SUM(F6:F7)</f>
         <v>800000</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="3">
         <f>SUM(G6:G7)</f>
         <v>720000</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="3">
         <f>SUM(H6:H7)</f>
         <v>805000</v>
       </c>
-      <c r="I5" s="21">
+      <c r="I5" s="19">
         <f>E5-H5</f>
         <v>-5000</v>
       </c>
-      <c r="J5" s="17">
+      <c r="J5" s="15">
         <f>SUMPRODUCT(E6:E7, J6:J7)/SUM(E6:E7)</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="5">
         <v>540000</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="7">
+      <c r="D6" s="12"/>
+      <c r="E6" s="5">
         <f t="shared" ref="E6:E26" si="0">SUM(C6:D6)</f>
         <v>540000</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="5">
         <v>540000</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="5">
         <v>486000</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="5">
         <v>540000</v>
       </c>
-      <c r="I6" s="22">
+      <c r="I6" s="20">
         <f t="shared" ref="I6:I27" si="1">E6-H6</f>
         <v>0</v>
       </c>
-      <c r="J6" s="18">
+      <c r="J6" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="6">
         <v>260000</v>
       </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="8">
+      <c r="D7" s="13"/>
+      <c r="E7" s="6">
         <f t="shared" si="0"/>
         <v>260000</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="6">
         <v>260000</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="6">
         <v>234000</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="6">
         <v>265000</v>
       </c>
-      <c r="I7" s="23">
+      <c r="I7" s="21">
         <f t="shared" si="1"/>
         <v>-5000</v>
       </c>
-      <c r="J7" s="19">
+      <c r="J7" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="3">
         <f>SUM(C9:C14)</f>
         <v>4290000</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="11">
         <f>SUM(D9:D14)</f>
         <v>45000</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="3">
         <f t="shared" si="0"/>
         <v>4335000</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="3">
         <f>SUM(F9:F14)</f>
         <v>4121000</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="3">
         <f>SUM(G9:G14)</f>
         <v>3708950</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="3">
         <f>SUM(H9:H14)</f>
         <v>4315000</v>
       </c>
-      <c r="I8" s="21">
+      <c r="I8" s="19">
         <f t="shared" si="1"/>
         <v>20000</v>
       </c>
-      <c r="J8" s="17">
+      <c r="J8" s="15">
         <f>SUMPRODUCT(E9:E14,J9:J14)/SUM(E9:E14)</f>
         <v>0.92612456747404848</v>
       </c>
     </row>
     <row r="9" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="5">
         <v>1800000</v>
       </c>
-      <c r="D9" s="14"/>
-      <c r="E9" s="7">
+      <c r="D9" s="12"/>
+      <c r="E9" s="5">
         <f t="shared" si="0"/>
         <v>1800000</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="5">
         <v>1800000</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="5">
         <v>1620000</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="5">
         <v>1800000</v>
       </c>
-      <c r="I9" s="22">
+      <c r="I9" s="20">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J9" s="18">
+      <c r="J9" s="16">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="6">
         <v>650000</v>
       </c>
-      <c r="D10" s="15"/>
-      <c r="E10" s="8">
+      <c r="D10" s="13"/>
+      <c r="E10" s="6">
         <f t="shared" si="0"/>
         <v>650000</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="6">
         <v>650000</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="6">
         <v>585000</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10" s="6">
         <v>650000</v>
       </c>
-      <c r="I10" s="23">
+      <c r="I10" s="21">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J10" s="19">
+      <c r="J10" s="17">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="5">
         <v>280000</v>
       </c>
-      <c r="D11" s="14"/>
-      <c r="E11" s="7">
+      <c r="D11" s="12"/>
+      <c r="E11" s="5">
         <f t="shared" si="0"/>
         <v>280000</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="5">
         <v>266000</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="5">
         <v>239400</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="5">
         <v>272000</v>
       </c>
-      <c r="I11" s="22">
+      <c r="I11" s="20">
         <f t="shared" si="1"/>
         <v>8000</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="16">
         <v>0.95</v>
       </c>
     </row>
     <row r="12" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="6">
         <v>950000</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="13">
         <v>45000</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="6">
         <f t="shared" si="0"/>
         <v>995000</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="6">
         <v>895500</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="6">
         <v>806000</v>
       </c>
-      <c r="H12" s="8">
+      <c r="H12" s="6">
         <v>1045000</v>
       </c>
-      <c r="I12" s="23">
+      <c r="I12" s="21">
         <f t="shared" si="1"/>
         <v>-50000</v>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="17">
         <v>0.85</v>
       </c>
     </row>
     <row r="13" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="5">
         <v>520000</v>
       </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="7">
+      <c r="D13" s="12"/>
+      <c r="E13" s="5">
         <f t="shared" si="0"/>
         <v>520000</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="5">
         <v>442000</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="5">
         <v>397800</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="5">
         <v>476000</v>
       </c>
-      <c r="I13" s="22">
+      <c r="I13" s="20">
         <f t="shared" si="1"/>
         <v>44000</v>
       </c>
-      <c r="J13" s="18">
+      <c r="J13" s="16">
         <v>0.75</v>
       </c>
     </row>
     <row r="14" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="6">
         <v>90000</v>
       </c>
-      <c r="D14" s="15"/>
-      <c r="E14" s="8">
+      <c r="D14" s="13"/>
+      <c r="E14" s="6">
         <f t="shared" si="0"/>
         <v>90000</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="6">
         <v>67500</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="6">
         <v>60750</v>
       </c>
-      <c r="H14" s="8">
+      <c r="H14" s="6">
         <v>72000</v>
       </c>
-      <c r="I14" s="23">
+      <c r="I14" s="21">
         <f t="shared" si="1"/>
         <v>18000</v>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="17">
         <v>0.7</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="3">
         <f>SUM(C16:C18)</f>
         <v>790000</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="11">
         <f>SUM(D16:D18)</f>
         <v>28000</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="3">
         <f t="shared" si="0"/>
         <v>818000</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="3">
         <f>SUM(F16:F18)</f>
         <v>626500</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="3">
         <f>SUM(G16:G18)</f>
         <v>501200</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="3">
         <f>SUM(H16:H18)</f>
         <v>842000</v>
       </c>
-      <c r="I15" s="21">
+      <c r="I15" s="19">
         <f t="shared" si="1"/>
         <v>-24000</v>
       </c>
-      <c r="J15" s="17">
+      <c r="J15" s="15">
         <f>SUMPRODUCT(E16:E18,J16:J18)/SUM(E16:E18)</f>
         <v>0.61589242053789728</v>
       </c>
     </row>
     <row r="16" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="5">
         <v>380000</v>
       </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="7">
+      <c r="D16" s="12"/>
+      <c r="E16" s="5">
         <f t="shared" si="0"/>
         <v>380000</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="5">
         <v>304000</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="5">
         <v>243200</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="5">
         <v>391000</v>
       </c>
-      <c r="I16" s="22">
+      <c r="I16" s="20">
         <f t="shared" si="1"/>
         <v>-11000</v>
       </c>
-      <c r="J16" s="18">
+      <c r="J16" s="16">
         <v>0.65</v>
       </c>
     </row>
     <row r="17" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="6">
         <v>290000</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="13">
         <v>28000</v>
       </c>
-      <c r="E17" s="8">
+      <c r="E17" s="6">
         <f t="shared" si="0"/>
         <v>318000</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="6">
         <v>238500</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="6">
         <v>190800</v>
       </c>
-      <c r="H17" s="8">
+      <c r="H17" s="6">
         <v>325000</v>
       </c>
-      <c r="I17" s="23">
+      <c r="I17" s="21">
         <f t="shared" si="1"/>
         <v>-7000</v>
       </c>
-      <c r="J17" s="19">
+      <c r="J17" s="17">
         <v>0.6</v>
       </c>
     </row>
     <row r="18" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="5">
         <v>120000</v>
       </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="7">
+      <c r="D18" s="12"/>
+      <c r="E18" s="5">
         <f t="shared" si="0"/>
         <v>120000</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="5">
         <v>84000</v>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="5">
         <v>67200</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="5">
         <v>126000</v>
       </c>
-      <c r="I18" s="22">
+      <c r="I18" s="20">
         <f t="shared" si="1"/>
         <v>-6000</v>
       </c>
-      <c r="J18" s="18">
+      <c r="J18" s="16">
         <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="3">
         <v>680000</v>
       </c>
-      <c r="D19" s="13"/>
-      <c r="E19" s="5">
+      <c r="D19" s="11"/>
+      <c r="E19" s="3">
         <f t="shared" si="0"/>
         <v>680000</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="3">
         <v>476000</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="3">
         <v>380800</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="3">
         <v>695000</v>
       </c>
-      <c r="I19" s="21">
+      <c r="I19" s="19">
         <f t="shared" si="1"/>
         <v>-15000</v>
       </c>
-      <c r="J19" s="17">
+      <c r="J19" s="15">
         <v>0.6</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="3">
         <f>SUM(C21:C23)</f>
         <v>7030000</v>
       </c>
-      <c r="D20" s="13">
+      <c r="D20" s="11">
         <f>SUM(D21:D23)</f>
         <v>157000</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="3">
         <f t="shared" si="0"/>
         <v>7187000</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="3">
         <f>SUM(F21:F23)</f>
         <v>6752050</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="3">
         <f>SUM(G21:G23)</f>
         <v>5403200</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="3">
         <f>SUM(H21:H23)</f>
         <v>7484000</v>
       </c>
-      <c r="I20" s="21">
+      <c r="I20" s="19">
         <f t="shared" si="1"/>
         <v>-297000</v>
       </c>
-      <c r="J20" s="17">
+      <c r="J20" s="15">
         <f>SUMPRODUCT(E21:E23,J21:J23)/SUM(E21:E23)</f>
         <v>0.66268262139974954</v>
       </c>
     </row>
     <row r="21" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="5">
         <v>3240000</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="12">
         <v>95000</v>
       </c>
-      <c r="E21" s="7">
+      <c r="E21" s="5">
         <f t="shared" si="0"/>
         <v>3335000</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="5">
         <v>3168250</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="5">
         <v>2534600</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="5">
         <v>3480000</v>
       </c>
-      <c r="I21" s="22">
+      <c r="I21" s="20">
         <f t="shared" si="1"/>
         <v>-145000</v>
       </c>
-      <c r="J21" s="18">
+      <c r="J21" s="16">
         <v>0.7</v>
       </c>
     </row>
     <row r="22" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="6">
         <v>2340000</v>
       </c>
-      <c r="D22" s="15"/>
-      <c r="E22" s="8">
+      <c r="D22" s="13"/>
+      <c r="E22" s="6">
         <f t="shared" si="0"/>
         <v>2340000</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="6">
         <v>2223000</v>
       </c>
-      <c r="G22" s="8">
+      <c r="G22" s="6">
         <v>1780000</v>
       </c>
-      <c r="H22" s="8">
+      <c r="H22" s="6">
         <v>2456000</v>
       </c>
-      <c r="I22" s="23">
+      <c r="I22" s="21">
         <f t="shared" si="1"/>
         <v>-116000</v>
       </c>
-      <c r="J22" s="19">
+      <c r="J22" s="17">
         <v>0.65</v>
       </c>
     </row>
     <row r="23" spans="1:10" outlineLevel="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="5">
         <v>1450000</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="12">
         <v>62000</v>
       </c>
-      <c r="E23" s="7">
+      <c r="E23" s="5">
         <f t="shared" si="0"/>
         <v>1512000</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="5">
         <v>1360800</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="5">
         <v>1088600</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="5">
         <v>1548000</v>
       </c>
-      <c r="I23" s="22">
+      <c r="I23" s="20">
         <f t="shared" si="1"/>
         <v>-36000</v>
       </c>
-      <c r="J23" s="18">
+      <c r="J23" s="16">
         <v>0.6</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="5">
+      <c r="C24" s="3">
         <v>600000</v>
       </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="5">
+      <c r="D24" s="11"/>
+      <c r="E24" s="3">
         <f t="shared" si="0"/>
         <v>600000</v>
       </c>
-      <c r="F24" s="5">
+      <c r="F24" s="3">
         <v>360000</v>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="3">
         <v>216000</v>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="3">
         <v>628000</v>
       </c>
-      <c r="I24" s="21">
+      <c r="I24" s="19">
         <f t="shared" si="1"/>
         <v>-28000</v>
       </c>
-      <c r="J24" s="17">
+      <c r="J24" s="15">
         <v>0.45</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="3">
         <v>2800000</v>
       </c>
-      <c r="D25" s="13">
+      <c r="D25" s="11">
         <v>85000</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="3">
         <f t="shared" si="0"/>
         <v>2885000</v>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="3">
         <v>2885000</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="3">
         <v>2596500</v>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="3">
         <v>3100000</v>
       </c>
-      <c r="I25" s="21">
+      <c r="I25" s="19">
         <f t="shared" si="1"/>
         <v>-215000</v>
       </c>
-      <c r="J25" s="17">
+      <c r="J25" s="15">
         <v>0.65</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="3">
         <v>1010000</v>
       </c>
-      <c r="D26" s="13"/>
-      <c r="E26" s="5">
+      <c r="D26" s="11"/>
+      <c r="E26" s="3">
         <f t="shared" si="0"/>
         <v>1010000</v>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="3">
         <v>0</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="3">
         <v>0</v>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="3">
         <v>850000</v>
       </c>
-      <c r="I26" s="21">
+      <c r="I26" s="19">
         <f t="shared" si="1"/>
         <v>160000</v>
       </c>
-      <c r="J26" s="17">
+      <c r="J26" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="6">
+      <c r="C27" s="4">
         <f t="shared" ref="C27:H27" si="2">SUM(C5,C8,C15,C19,C20,C24,C25,C26)</f>
         <v>18000000</v>
       </c>
-      <c r="D27" s="16">
+      <c r="D27" s="14">
         <f t="shared" si="2"/>
         <v>315000</v>
       </c>
-      <c r="E27" s="16">
+      <c r="E27" s="14">
         <f t="shared" si="2"/>
         <v>18315000</v>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="4">
         <f t="shared" si="2"/>
         <v>16020550</v>
       </c>
-      <c r="G27" s="6">
+      <c r="G27" s="4">
         <f t="shared" si="2"/>
         <v>13526650</v>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="4">
         <f t="shared" si="2"/>
         <v>18719000</v>
       </c>
-      <c r="I27" s="24">
+      <c r="I27" s="22">
         <f t="shared" si="1"/>
         <v>-404000</v>
       </c>
-      <c r="J27" s="20">
+      <c r="J27" s="18">
         <f>SUMPRODUCT(E5:E26,J5:J26)/SUM(E5:E26)</f>
         <v>0.72216658718804638</v>
       </c>
@@ -3050,13 +3060,13 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:I27">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>AND(I5&lt;0, I5&gt;=-E5*0.02)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3080,208 +3090,208 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
     </row>
     <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="41" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="43" t="s">
+      <c r="D4" s="41" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="41" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="43" t="s">
+      <c r="F4" s="41" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="44" t="s">
+      <c r="G4" s="42" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A5" s="25">
+      <c r="A5" s="23">
         <v>45383</v>
       </c>
-      <c r="B5" s="26">
+      <c r="B5" s="24">
         <v>850000</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="24">
         <v>820000</v>
       </c>
-      <c r="D5" s="45">
+      <c r="D5" s="43">
         <f>B5-C5</f>
         <v>30000</v>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="25">
         <f>D5/B5</f>
         <v>3.5294117647058823E-2</v>
       </c>
-      <c r="F5" s="28">
+      <c r="F5" s="26">
         <f>B5/C5</f>
         <v>1.0365853658536586</v>
       </c>
-      <c r="G5" s="29">
+      <c r="G5" s="27">
         <f>18315000/F5</f>
         <v>17668588.235294119</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A6" s="30">
+      <c r="A6" s="28">
         <v>45413</v>
       </c>
-      <c r="B6" s="31">
+      <c r="B6" s="29">
         <v>1920000</v>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="29">
         <v>1850000</v>
       </c>
-      <c r="D6" s="46">
+      <c r="D6" s="44">
         <f t="shared" ref="D6:D10" si="0">B6-C6</f>
         <v>70000</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="30">
         <f t="shared" ref="E6:E10" si="1">D6/B6</f>
         <v>3.6458333333333336E-2</v>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="31">
         <f t="shared" ref="F6:F10" si="2">B6/C6</f>
         <v>1.0378378378378379</v>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="32">
         <f t="shared" ref="G6:G10" si="3">18315000/F6</f>
         <v>17647265.625</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A7" s="25">
+      <c r="A7" s="23">
         <v>45444</v>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="24">
         <v>3450000</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="24">
         <v>3350000</v>
       </c>
-      <c r="D7" s="45">
+      <c r="D7" s="43">
         <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="25">
         <f t="shared" si="1"/>
         <v>2.8985507246376812E-2</v>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="26">
         <f t="shared" si="2"/>
         <v>1.0298507462686568</v>
       </c>
-      <c r="G7" s="29">
+      <c r="G7" s="27">
         <f t="shared" si="3"/>
         <v>17784130.434782606</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A8" s="30">
+      <c r="A8" s="28">
         <v>45474</v>
       </c>
-      <c r="B8" s="31">
+      <c r="B8" s="29">
         <v>5280000</v>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="29">
         <v>5180000</v>
       </c>
-      <c r="D8" s="46">
+      <c r="D8" s="44">
         <f t="shared" si="0"/>
         <v>100000</v>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="30">
         <f t="shared" si="1"/>
         <v>1.893939393939394E-2</v>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="31">
         <f t="shared" si="2"/>
         <v>1.0193050193050193</v>
       </c>
-      <c r="G8" s="34">
+      <c r="G8" s="32">
         <f t="shared" si="3"/>
         <v>17968125</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A9" s="25">
+      <c r="A9" s="23">
         <v>45505</v>
       </c>
-      <c r="B9" s="26">
+      <c r="B9" s="24">
         <v>8640000</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="24">
         <v>8750000</v>
       </c>
-      <c r="D9" s="45">
+      <c r="D9" s="43">
         <f t="shared" si="0"/>
         <v>-110000</v>
       </c>
-      <c r="E9" s="27">
+      <c r="E9" s="25">
         <f t="shared" si="1"/>
         <v>-1.2731481481481481E-2</v>
       </c>
-      <c r="F9" s="28">
+      <c r="F9" s="26">
         <f t="shared" si="2"/>
         <v>0.98742857142857143</v>
       </c>
-      <c r="G9" s="29">
+      <c r="G9" s="27">
         <f t="shared" si="3"/>
         <v>18548177.083333332</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A10" s="35">
+      <c r="A10" s="33">
         <v>45536</v>
       </c>
-      <c r="B10" s="36">
+      <c r="B10" s="34">
         <v>11850000</v>
       </c>
-      <c r="C10" s="36">
+      <c r="C10" s="34">
         <v>12254650</v>
       </c>
-      <c r="D10" s="47">
+      <c r="D10" s="45">
         <f t="shared" si="0"/>
         <v>-404650</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="35">
         <f t="shared" si="1"/>
         <v>-3.4147679324894514E-2</v>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="36">
         <f t="shared" si="2"/>
         <v>0.96697988110635558</v>
       </c>
-      <c r="G10" s="39">
+      <c r="G10" s="37">
         <f t="shared" si="3"/>
         <v>18940414.746835444</v>
       </c>
@@ -3302,10 +3312,10 @@
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="D5:D10">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>D5&lt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>D5&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3324,74 +3334,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="48" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="49" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="48" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
+      <c r="A4" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="50">
         <v>18000000</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
+      <c r="A5" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="51">
         <v>45383</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
+      <c r="A6" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="52">
         <v>46112</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
+      <c r="A7" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="48" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
+      <c r="A8" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="49" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
+      <c r="A9" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="48">
         <v>0.65</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add Government Office Refurbishment cost plan and CVR
</commit_message>
<xml_diff>
--- a/cost-plans/NHS-Acute-Hospital-Wing.xlsx
+++ b/cost-plans/NHS-Acute-Hospital-Wing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C802EC-DCA2-414A-97D1-74503BD634BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA05768E-2A77-4889-A3C5-DD503497D0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="2" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="1" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Plan" sheetId="1" r:id="rId1"/>
@@ -284,8 +284,8 @@
   <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="171" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="174" formatCode="&quot;£&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="&quot;£&quot;#,##0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -513,26 +513,20 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="17" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="5" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -541,20 +535,26 @@
     <xf numFmtId="38" fontId="0" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="174" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -564,18 +564,6 @@
     <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="5">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF70AD47"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -617,6 +605,18 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF70AD47"/>
         </patternFill>
       </fill>
     </dxf>
@@ -709,7 +709,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -843,22 +843,22 @@
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>45383</c:v>
+                  <c:v>45931</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>45413</c:v>
+                  <c:v>45962</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>45444</c:v>
+                  <c:v>45992</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45474</c:v>
+                  <c:v>46023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45505</c:v>
+                  <c:v>46054</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>45536</c:v>
+                  <c:v>46082</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1021,22 +1021,22 @@
                 <c:formatCode>mmm\-yy</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>45383</c:v>
+                  <c:v>45931</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>45413</c:v>
+                  <c:v>45962</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>45444</c:v>
+                  <c:v>45992</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45474</c:v>
+                  <c:v>46023</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>45505</c:v>
+                  <c:v>46054</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>45536</c:v>
+                  <c:v>46082</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2214,33 +2214,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
     </row>
     <row r="2" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="39" t="str">
+      <c r="A2" s="52" t="str">
         <f ca="1">"Meridian Cost Consultants | Report Date: "&amp;TEXT(TODAY(),"DD MMMM YYYY")</f>
-        <v>Meridian Cost Consultants | Report Date: 13 May 2026</v>
-      </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
+        <v>Meridian Cost Consultants | Report Date: 15 May 2026</v>
+      </c>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="7" t="s">
@@ -3060,13 +3060,13 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:I27">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>AND(I5&lt;0, I5&gt;=-E5*0.02)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3090,53 +3090,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="51" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="52" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
     </row>
     <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="39" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="39" t="s">
         <v>74</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="39" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="G4" s="42" t="s">
+      <c r="G4" s="40" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="23">
-        <v>45383</v>
+        <v>45931</v>
       </c>
       <c r="B5" s="24">
         <v>850000</v>
@@ -3144,7 +3144,7 @@
       <c r="C5" s="24">
         <v>820000</v>
       </c>
-      <c r="D5" s="43">
+      <c r="D5" s="41">
         <f>B5-C5</f>
         <v>30000</v>
       </c>
@@ -3163,7 +3163,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="28">
-        <v>45413</v>
+        <v>45962</v>
       </c>
       <c r="B6" s="29">
         <v>1920000</v>
@@ -3171,7 +3171,7 @@
       <c r="C6" s="29">
         <v>1850000</v>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="42">
         <f t="shared" ref="D6:D10" si="0">B6-C6</f>
         <v>70000</v>
       </c>
@@ -3190,7 +3190,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="23">
-        <v>45444</v>
+        <v>45992</v>
       </c>
       <c r="B7" s="24">
         <v>3450000</v>
@@ -3198,7 +3198,7 @@
       <c r="C7" s="24">
         <v>3350000</v>
       </c>
-      <c r="D7" s="43">
+      <c r="D7" s="41">
         <f t="shared" si="0"/>
         <v>100000</v>
       </c>
@@ -3217,7 +3217,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="28">
-        <v>45474</v>
+        <v>46023</v>
       </c>
       <c r="B8" s="29">
         <v>5280000</v>
@@ -3225,7 +3225,7 @@
       <c r="C8" s="29">
         <v>5180000</v>
       </c>
-      <c r="D8" s="44">
+      <c r="D8" s="42">
         <f t="shared" si="0"/>
         <v>100000</v>
       </c>
@@ -3244,7 +3244,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="23">
-        <v>45505</v>
+        <v>46054</v>
       </c>
       <c r="B9" s="24">
         <v>8640000</v>
@@ -3252,7 +3252,7 @@
       <c r="C9" s="24">
         <v>8750000</v>
       </c>
-      <c r="D9" s="43">
+      <c r="D9" s="41">
         <f t="shared" si="0"/>
         <v>-110000</v>
       </c>
@@ -3271,7 +3271,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="33">
-        <v>45536</v>
+        <v>46082</v>
       </c>
       <c r="B10" s="34">
         <v>11850000</v>
@@ -3279,7 +3279,7 @@
       <c r="C10" s="34">
         <v>12254650</v>
       </c>
-      <c r="D10" s="45">
+      <c r="D10" s="43">
         <f t="shared" si="0"/>
         <v>-404650</v>
       </c>
@@ -3312,11 +3312,11 @@
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="D5:D10">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>D5&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>D5&lt;0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>D5&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3334,74 +3334,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="46" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="49" t="s">
+      <c r="B2" s="47" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="48" t="s">
+      <c r="B3" s="46" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="50">
+      <c r="B4" s="48">
         <v>18000000</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="51">
+      <c r="B5" s="49">
         <v>45383</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="52">
+      <c r="B6" s="50">
         <v>46112</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A7" s="46" t="s">
+      <c r="A7" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="46" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A8" s="47" t="s">
+      <c r="A8" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="49" t="s">
+      <c r="B8" s="47" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A9" s="46" t="s">
+      <c r="A9" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="48">
+      <c r="B9" s="46">
         <v>0.65</v>
       </c>
     </row>

</xml_diff>